<commit_message>
Correct MPE description and assembly-factor titles, add 06 README
</commit_message>
<xml_diff>
--- a/05_Mitochondria/01_build_mito_sets/c_data/01_build_mito_sets.xlsx
+++ b/05_Mitochondria/01_build_mito_sets/c_data/01_build_mito_sets.xlsx
@@ -7,8 +7,7 @@
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
-    <sheet name="overview" sheetId="1" r:id="rId1"/>
-    <sheet name="membership" sheetId="2" r:id="rId2"/>
+    <sheet name="membership" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -352,48 +351,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>sheet</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>rows</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>membership</t>
-        </is>
-      </c>
-      <c r="B2">
-        <v>5040</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>One row per set and gene, flagged if measured. 02_test_mito reads this sheet.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D5041"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>

</xml_diff>